<commit_message>
Refresh sample inputs through Profiler v01.4 (27-screen + value-based tier)
Replayed each sample's own answer codes through the current Profiler so the
exports reflect v01.4 and the value-based tier fix. Profiles preserved
(AB2123 VC76, Copilot VC18). Verified end-to-end in Autogenerate: both still
generate (AB2123 needs 6 templates / 26 generate=Y after moving up to Full;
Copilot 5 / 16), full handoff intact (Templates/Fields/Loops/CA-PMF/
Contradictions), security fires.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019cfSkM9c5hauJaK734DdoX
</commit_message>
<xml_diff>
--- a/tier-unification/sample-inputs/SAMPLE_Profiler-Export_Copilot-Pilot_MINI_VC18.xlsx
+++ b/tier-unification/sample-inputs/SAMPLE_Profiler-Export_Copilot-Pilot_MINI_VC18.xlsx
@@ -1890,7 +1890,7 @@
     </row>
     <row r="28">
       <c r="A28" s="12" t="str">
-        <v>EDD · ESPMO Project Profiler   ·   Licenses for GitHub Copilot Pilot   ·   Sheet 1 of 8   ·   Generated Jul 2, 2026</v>
+        <v>EDD · ESPMO Project Profiler   ·   Licenses for GitHub Copilot Pilot   ·   Sheet 1 of 8   ·   Generated Jul 6, 2026</v>
       </c>
       <c r="B28" s="12" t="str">
         <v/>
@@ -2057,7 +2057,7 @@
         <v>version</v>
       </c>
       <c r="B18" s="2" t="str">
-        <v>v01.07</v>
+        <v>v01.09</v>
       </c>
     </row>
     <row r="19">
@@ -2065,7 +2065,7 @@
         <v>generated_on</v>
       </c>
       <c r="B19" s="2" t="str">
-        <v>2026-07-02</v>
+        <v>2026-07-06</v>
       </c>
     </row>
     <row r="20">
@@ -4754,7 +4754,7 @@
     </row>
     <row r="35">
       <c r="A35" s="12" t="str">
-        <v>EDD · ESPMO Project Profiler   ·   Licenses for GitHub Copilot Pilot   ·   Sheet 2 of 8   ·   Generated Jul 2, 2026</v>
+        <v>EDD · ESPMO Project Profiler   ·   Licenses for GitHub Copilot Pilot   ·   Sheet 2 of 8   ·   Generated Jul 6, 2026</v>
       </c>
       <c r="B35" s="12" t="str">
         <v/>
@@ -6350,7 +6350,7 @@
     </row>
     <row r="44">
       <c r="A44" s="12" t="str">
-        <v>EDD · ESPMO Project Profiler   ·   Licenses for GitHub Copilot Pilot   ·   Sheet 4 of 8   ·   Generated Jul 2, 2026</v>
+        <v>EDD · ESPMO Project Profiler   ·   Licenses for GitHub Copilot Pilot   ·   Sheet 4 of 8   ·   Generated Jul 6, 2026</v>
       </c>
       <c r="B44" s="12" t="str">
         <v/>
@@ -7455,7 +7455,7 @@
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="12" t="str">
-        <v>EDD · ESPMO Project Profiler   ·   Licenses for GitHub Copilot Pilot   ·   Sheet 5 of 8   ·   Generated Jul 2, 2026</v>
+        <v>EDD · ESPMO Project Profiler   ·   Licenses for GitHub Copilot Pilot   ·   Sheet 5 of 8   ·   Generated Jul 6, 2026</v>
       </c>
       <c r="B38" s="12" t="str">
         <v/>
@@ -8885,7 +8885,7 @@
     </row>
     <row r="48" ht="16" customHeight="1">
       <c r="A48" s="12" t="str">
-        <v>EDD · ESPMO Project Profiler   ·   Licenses for GitHub Copilot Pilot   ·   Sheet 7 of 8   ·   Generated Jul 2, 2026</v>
+        <v>EDD · ESPMO Project Profiler   ·   Licenses for GitHub Copilot Pilot   ·   Sheet 7 of 8   ·   Generated Jul 6, 2026</v>
       </c>
       <c r="B48" s="12" t="str">
         <v/>
@@ -9999,7 +9999,7 @@
     </row>
     <row r="49">
       <c r="A49" s="12" t="str">
-        <v>EDD · ESPMO Project Profiler   ·   Licenses for GitHub Copilot Pilot   ·   Sheet 8 of 8   ·   Generated Jul 2, 2026</v>
+        <v>EDD · ESPMO Project Profiler   ·   Licenses for GitHub Copilot Pilot   ·   Sheet 8 of 8   ·   Generated Jul 6, 2026</v>
       </c>
       <c r="B49" s="12" t="str">
         <v/>

</xml_diff>